<commit_message>
build(track2-it1): the PDF and the xlsx re-rendered from the restructured sources
Rebuilt with the folder README's own "Regenerate this folder" commands
(tools/md_to_html.py then node tools/md_to_pdf.mjs; tools/fill_methods_form.py
on the Track 2 methods sheet). Gates: check_iteration reports "draft - ok",
check_coordinates reports clean.
</commit_message>
<xml_diff>
--- a/submissions/track2/iteration-1/agharsallah_track2_methods_form.xlsx
+++ b/submissions/track2/iteration-1/agharsallah_track2_methods_form.xlsx
@@ -679,7 +679,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>From variant to mechanism to medicine in four documented stages, each a case-agnostic tool with a provenance manifest. (1) Hand-off: Track 1's confirmed compound-heterozygous BUB1B pair (a stop allele + a kinase-region missense, trans configuration confirmed by the challenge's answer key) was written into a structured 'mechanism card' (ressources/track2/mechanism.json): gene, protein, the two allele classes (never positions), loss-of-function reading, the spindle-assembly-checkpoint pathway, downstream consequences, the tumour context (rhabdomyosarcoma) from the clinical terms, and four repurposing directions with seed genes - D1 reinforce the checkpoint, D2 exploit aneuploidy stress, D3 stabilise the remaining BubR1 (hypomorph), D4 the child's tumour. Iteration 2's measured genotype facts (allele dosage from the raw reads, exon copy number, structural-variant absence, the missense's position in the protein, pathogenicity lanes, P(trans)) were appended as a card revision (v3), with the aneuploidy burden marked unmeasured. (2) Search: the card's seeds were expanded through Reactome pathways to 277 targets; Open Targets, ChEMBL and DGIdb returned 3,859 drug-target rows and 359 market-approved drugs; openFDA confirmed US labels; ClinicalTrials.gov and PubMed answered trial and literature questions, all queries derived from the card. (3) Grading: every approved drug on every direction was placed on a five-rung evidence ladder pre-registered before the search (5 approved for a related indication with paediatric use; 4 trial in a related indication; 3 animal model of the mechanism; 2 cell model; 1 mechanism only - named, never submitted). Automated tests (approval, label and its Pediatric Use section, tumour-context trials, studies admitting children, PubMed co-mention counts) and curated tests (one PubMed paper per row, read by a person, 13 rows) are printed side by side; inherited class-level evidence is marked 'proxy'. Six falsifiable claims (one per direction, one for the control, one for paediatric data) were registered with predictions and refutation conditions before any drug-level query. (4) Control: the same pipeline ran on two decoy cards - the child's clinical side kept, the gene swapped (NTRK3 by a seeded draw from Track 1's decoy set; XDH, an unrelated metabolic enzyme). A direction whose approved drugs overlap a decoy's at Jaccard &gt;= 0.10 is reported as non-specific; D4 did (0.25) and is argued only from curated mechanism results. Output: 11 drugs with a cited mechanism result (statins; niacin/nicotinamide; chloroquine; bortezomib, metformin, valproic acid, vorinostat, hydroxychloroquine, atorvastatin), 50 drugs already in rhabdomyosarcoma trials listed as such, and a 23-drug do-not table (spindle poisons, checkpoint inhibitors, standard of care).</t>
+          <t>From variant to mechanism to medicine in four documented stages, each a case-agnostic tool with a provenance manifest. (1) Hand-off: Track 1's confirmed compound-heterozygous BUB1B pair (a stop allele + a kinase-region missense, trans configuration confirmed by the challenge's answer key) was written into a structured 'mechanism card' (ressources/track2/mechanism.json): gene, protein, the two allele classes (never positions), loss-of-function reading, the spindle-assembly-checkpoint pathway, downstream consequences, the tumour context (rhabdomyosarcoma) from the clinical terms, and four repurposing directions with seed genes - D1 reinforce the checkpoint, D2 exploit aneuploidy stress, D3 stabilise the remaining BubR1 (hypomorph), D4 the child's tumour. Iteration 2's measured genotype facts (allele dosage from the raw reads, exon copy number, structural-variant absence, the missense's position in the protein, pathogenicity lanes, P(trans)) were appended as a card revision (v3), with the aneuploidy burden marked unmeasured. (2) Search: the card's seeds were expanded through Reactome pathways to 277 targets; Open Targets, ChEMBL and DGIdb returned 3,859 drug-target rows and 359 market-approved drugs; openFDA confirmed US labels; ClinicalTrials.gov and PubMed answered trial and literature questions, all queries derived from the card. (3) Grading: every approved drug on every direction was placed on a five-rung evidence ladder pre-registered before the search (5 approved for a related indication with paediatric use; 4 trial in a related indication; 3 animal model of the mechanism; 2 cell model; 1 mechanism only - named, never submitted). Automated tests (approval, label and its Pediatric Use section, tumour-context trials, studies admitting children, PubMed co-mention counts) and curated tests (one PubMed paper per row, read by a person, 13 rows) are printed side by side; inherited class-level evidence is marked 'proxy'. Six falsifiable claims (one per direction, one for the control, one for paediatric data) were registered with predictions and refutation conditions before any drug-level query. (4) Control: the same pipeline ran on two decoy cards - the child's clinical side kept, the gene swapped (NTRK3 by a seeded draw from Track 1's decoy set; XDH, an unrelated metabolic enzyme). This is a negative control in the usual sense: an input the pipeline should not be able to argue from, run through the unchanged code so that whatever comes out for the decoy as readily as for BUB1B is attributed to database density or the clinical queries rather than to the mechanism. A direction whose approved drugs overlap a decoy's at Jaccard &gt;= 0.10 is reported as non-specific; D4 did (0.25) and is argued only from curated mechanism results. Output: 11 drugs with a cited mechanism result (statins; niacin/nicotinamide; chloroquine; bortezomib, metformin, valproic acid, vorinostat, hydroxychloroquine, atorvastatin), 50 drugs already in rhabdomyosarcoma trials listed as such, and a 23-drug do-not table (spindle poisons, checkpoint inhibitors, standard of care).</t>
         </is>
       </c>
     </row>
@@ -763,7 +763,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Roughly four working days across two people-equivalents: one day for the mechanism card and the data layer (iteration 1, 2026-09-05/06), and about three days on 2026-09-18 for the card revision, the six pre-registered claims, the enrichment adapters and ladder, the decoy control, the curation, the figures, the dashboard page and this report. Compute: two laptop runs of about ten minutes each against public APIs; no cloud.</t>
+          <t>Roughly four working days across two people-equivalents: one day for the mechanism card and the data layer (iteration 1, 2026-09-05/06), and about three days on 2026-09-18 for the card revision, the six pre-registered claims, the enrichment adapters and ladder, the decoy control, the curation, the figures, the dashboard page and this report. Compute and cost: a laptop, two runs of about ten minutes each (the snapshot and the enrichment) against seven public APIs, most of that runtime spent waiting politely between per-drug requests rather than computing; seconds on a re-run once the replies are cached. No cloud, no GPU, no cluster, no paid data source and no licence fee - the only cost that does not shrink on a second case is the person-read curation (13 abstracts, one reader, one day).</t>
         </is>
       </c>
     </row>

</xml_diff>